<commit_message>
docs(AdminApp): Batch 6 — class grade settings / clone / context (81 TCs, all 30 scenarios)
Adds the final 13 TCs to the Classes-tab manual test-case suite, completing coverage
of every AdminApp.xlsx scenario:
- CGST (6): #22 class grade settings (Actions -> Class grade settings): grading scale,
  score settings, score calculation, weightage, add grading category, total 100%.
  Resolves the deferred launch [ASSUMED]s in GCAT_TC_7 / GSCL_TC_7.
- CLON (3): #31 clone via "Copy an Existing Class" (Teachers/materials/assignments/
  locked content rules/grade settings; empty components disabled).
- CTXC (4): #32 context class — [ASSUMED], no admin creation entry point found; needs
  teacher/student accounts + product clarification.

Numbering: unnumbered xlsx rows keyed by position (clone=#31, context=#32) to avoid
clashing with Batch-1 #28/#29 (ended-active, launch-from-ended). Suite now 81 TCs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/AdminApp-Classes/AdminApp_Classes_tab_test_cases.xlsx
@@ -5042,6 +5042,942 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">69</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CGST_TC_1</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the Class grade settings page launches from a class page</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#22 — Launch class grade setting page from a class page</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A class is open (Classes tab -&gt; launch a class).</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. On the class page, open the Actions menu. 2. Click Class grade settings.</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Class grade settings page opens (/class/.../grade-weighting) showing Grading Scale (+ Change), Score settings (teacher-override toggle), Score calculation (Best/First score), per-material Weightage %, Other grading categories (+ Add a grading category), Total grade: 100%, Save changes / Cancel.</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Destination the grading category/scale details pages link to (TST_GCAT_TC_7, TST_GSCL_TC_7).</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CGST_TC_2</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the grading scale can be changed for a class</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#22 — Launch class grade setting page from a class page</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the Class grade settings page.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. In Grading Scale, click Change. 2. Select a grading scale. 3. Click Save changes.</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A grading scale (AutoTest Scale / Cambridge One grading scale)</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Class grading scale updates to the selected scale; the class then appears under that scale's details. [ASSUMED] confirm change-scale selector.</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Associates a scale with a class - resolves TST_GSCL_TC_7.</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CGST_TC_3</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify a grading category can be added to a class</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#22 — Launch class grade setting page from a class page</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the Class grade settings page.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Click Add a grading category. 2. Select a grading category. 3. Set its Weightage %. 4. Click Save changes.</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A grading category (some) + weightage</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grading category added to the class with a weightage; the class then appears under that category's details. [ASSUMED] confirm add-category selector.</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Associates a category with a class - resolves TST_GCAT_TC_7.</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CGST_TC_4</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the score calculation (Best / First score) can be changed</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#22 — Launch class grade setting page from a class page</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the Class grade settings page.</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the Score calculation dropdown. 2. Select First score (or Best score). 3. Click Save changes.</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Score type: First score</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selected score type is saved as the score that counts toward students' progress.</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">73</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CGST_TC_5</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the teacher score-override setting can be toggled</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#22 — Launch class grade setting page from a class page</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the Class grade settings page.</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Toggle Allow teachers to override and add scores to auto-marked activities. 2. Click Save changes.</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The override setting is saved in the state it was toggled to.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CGST_TC_6</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the total grade weightage must equal 100%</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#22 — Launch class grade setting page from a class page</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the Class grade settings page with &gt;=1 material/category weightage.</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Set weightages that do not add up to 100%. 2. Attempt to Save changes.</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weightages summing to != 100%</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saving is prevented / an error shown until Total grade equals 100%. [ASSUMED] confirm validation copy.</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page shows a running Total grade: 100%.</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CLON_TC_1</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify a class can be cloned from an existing class</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#31 — Verify class clone functionality (Copy an Existing Class)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the Create new classes form with &gt;=1 row selected; a source class exists.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Click Copy an Existing Class. 2. Step 1: search and select the source class -&gt; Continue. 3. Step 2: on Choose what to copy from [source], select components -&gt; Continue.</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source class: SarthakTestClass1</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step 2 lists copyable components as checkboxes - Teachers, Course materials, Assignments, Locked content rules, Class grade settings - each with a count; selected components are copied from the source into the selected new row(s).</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Distinct from Duplicate (TST_BCCF_TC_7).</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">76</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CLON_TC_2</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify all components copy from a fully-populated source class</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#31 — Verify class clone functionality (Copy an Existing Class)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A source class that HAS a teacher, course materials, assignments, locked content rules (incl. an assignment-created lock rule), and class grade settings.</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Copy an Existing Class -&gt; select the populated source. 2. Select all available components. 3. Continue and create.</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A fully-populated source class [ASSUMED]</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The cloned class contains the source's teacher, materials, assignments, locked content rules (incl. the assignment-created rule), and class grade settings. [ASSUMED] verify each component copies (tested sources had 0 of each).</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requires a seeded source class.</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CLON_TC_3</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify components with no items are not selectable when copying</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#31 — Verify class clone functionality (Copy an Existing Class)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A source class that has 0 of one or more components.</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Copy an Existing Class -&gt; select a source with empty components -&gt; Continue.</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source: SarthakTestClass1 (0 teachers/materials/assignments/rules)</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Components with a count of 0 are disabled/unselectable (e.g. Teachers [0] disabled; Class grade settings - Not available).</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed live.</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CTXC_TC_1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify a context class can be created</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#32 — Verify Context class creation and view in teacher/admin/student login</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logged in as school admin. [ASSUMED] context-class creation path TBD.</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Create a context class via the (to-be-confirmed) context-class creation flow.</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Context class details [ASSUMED]</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The context class is created successfully. [ASSUMED] confirm the creation entry point and any context-specific fields.</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entry point not found in the admin bulk-create form; needs product clarification.</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">79</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CTXC_TC_2</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the context class appears in the admin login</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#32 — Verify Context class creation and view in teacher/admin/student login</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A context class exists; logged in as school admin.</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the school's Classes tab. 2. Locate the context class.</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The created context class</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The context class is listed and behaves as expected in the admin view. [ASSUMED] confirm admin-specific behaviour.</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CTXC_TC_3</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the context class appears/behaves correctly in the teacher login</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#32 — Verify Context class creation and view in teacher/admin/student login</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A context class exists; a teacher account associated with it.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Log in as the teacher. 2. Locate/open the context class.</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teacher account [ASSUMED]</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The context class is visible and behaves correctly for the teacher role. [ASSUMED] needs a teacher test account.</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-role verification.</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TST_CTXC_TC_4</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the context class appears/behaves correctly in the student login</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#32 — Verify Context class creation and view in teacher/admin/student login</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A context class exists; a student account enrolled in it.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Log in as the student. 2. Locate/open the context class.</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Student account [ASSUMED]</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The context class is visible and behaves correctly for the student role. [ASSUMED] needs a student test account.</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-role verification.</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>